<commit_message>
Rewrite all student-facing text in a plainer style
House style, now recorded in CONTRIBUTING-CONTENT.md: short sentences,
common words, no idioms, no commentary on the material itself, numbered
steps for instructions, and a full stop in place of a dash.

Rewritten: all five tutorial files, index, methodology and reference pages,
the checker and engine messages, the progress export, and the text inside
both Excel workbooks.

Measured over the tutorial prose: mean sentence length is now 10.8 words,
median 9, with 1.1% of sentences over 30 words. A scan for filler and
fourth-wall phrases returns nothing.

Every id, answer, tolerance, also_accept, correct flag and verify
expression is unchanged. All 341 answer checks and 332 browser checks pass,
and the workbench formulas still evaluate.
</commit_message>
<xml_diff>
--- a/data/xlsx/transport-stats-data.xlsx
+++ b/data/xlsx/transport-stats-data.xlsx
@@ -590,14 +590,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>On the travel time sheet the observations sit in B4:B58, so the cell</t>
+          <t>On the travel time sheet, the values are in B4:B58. The solutions in the</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>references used in the tutorial worked solutions apply exactly as written.</t>
+          <t>tutorials use this range.</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>The same data is available as CSV in data/csv/ if you prefer R or Python.</t>
+          <t>The same data is in data/csv/ as CSV files, for R and Python.</t>
         </is>
       </c>
     </row>

</xml_diff>